<commit_message>
feat(ui): Rebranding a FISCERTA, Tema cibernético Aurora y Proforma Clara
</commit_message>
<xml_diff>
--- a/Archivos_pruebas_2/M 2 PROFORMA MAGAÑA Y VIEIRA-CESMA_SERV. ASESORIA FIN. 5 de 24, Q1 MARZO 2026, MARTES 03.xlsx
+++ b/Archivos_pruebas_2/M 2 PROFORMA MAGAÑA Y VIEIRA-CESMA_SERV. ASESORIA FIN. 5 de 24, Q1 MARZO 2026, MARTES 03.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="10917"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="29725"/>
   <workbookPr autoCompressPictures="0"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/ricardo/Documents/0 Descargas apple/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Proyectos\Memoria\B2B_Materialidad\Archivos_pruebas_2\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3C2C5AF3-4863-2649-A56A-B762F0A3B36F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C83E6029-4F22-436C-99D4-060119662F18}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="2380" yWindow="960" windowWidth="23540" windowHeight="14980" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="366" yWindow="366" windowWidth="21390" windowHeight="11940" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="PROFORMA MVC CESAMA FINANCIERA" sheetId="4" r:id="rId1"/>
@@ -401,9 +401,6 @@
     <t xml:space="preserve">REQUIERE COTIZACION (S/N) </t>
   </si>
   <si>
-    <t>S</t>
-  </si>
-  <si>
     <t>REQUIRE CONTRATO (S/N)</t>
   </si>
   <si>
@@ -423,6 +420,9 @@
   </si>
   <si>
     <t>MVC151216BZ0</t>
+  </si>
+  <si>
+    <t>s</t>
   </si>
 </sst>
 </file>
@@ -430,9 +430,9 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
   <numFmts count="3">
-    <numFmt numFmtId="164" formatCode="_-&quot;$&quot;* #,##0.00_-;\-&quot;$&quot;* #,##0.00_-;_-&quot;$&quot;* &quot;-&quot;??_-;_-@_-"/>
-    <numFmt numFmtId="165" formatCode="[$-80A]d&quot; de &quot;mmmm&quot; de &quot;yyyy;@"/>
-    <numFmt numFmtId="166" formatCode="_-&quot;$&quot;* #,##0.0000_-;\-&quot;$&quot;* #,##0.0000_-;_-&quot;$&quot;* &quot;-&quot;??_-;_-@_-"/>
+    <numFmt numFmtId="44" formatCode="_-&quot;$&quot;* #,##0.00_-;\-&quot;$&quot;* #,##0.00_-;_-&quot;$&quot;* &quot;-&quot;??_-;_-@_-"/>
+    <numFmt numFmtId="164" formatCode="[$-80A]d&quot; de &quot;mmmm&quot; de &quot;yyyy;@"/>
+    <numFmt numFmtId="165" formatCode="_-&quot;$&quot;* #,##0.0000_-;\-&quot;$&quot;* #,##0.0000_-;_-&quot;$&quot;* &quot;-&quot;??_-;_-@_-"/>
   </numFmts>
   <fonts count="7" x14ac:knownFonts="1">
     <font>
@@ -730,7 +730,7 @@
   <cellStyleXfs count="3">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="0"/>
-    <xf numFmtId="164" fontId="6" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="44" fontId="6" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
   <cellXfs count="82">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
@@ -745,24 +745,171 @@
     <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
       <alignment vertical="top"/>
     </xf>
-    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="2" applyFont="1"/>
-    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="44" fontId="0" fillId="0" borderId="0" xfId="2" applyFont="1"/>
+    <xf numFmtId="44" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="166" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="165" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="4" fontId="0" fillId="2" borderId="1" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
+    <xf numFmtId="49" fontId="4" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="1" fillId="3" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="1" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="13" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="14" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="15" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="16" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="17" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="18" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="19" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="20" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="2" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="3" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="4" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="49" fontId="4" fillId="0" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="49" fontId="4" fillId="0" borderId="8" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="49" fontId="4" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="49" fontId="4" fillId="0" borderId="12" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="49" fontId="4" fillId="0" borderId="6" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="49" fontId="4" fillId="0" borderId="11" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="44" fontId="0" fillId="2" borderId="2" xfId="2" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="44" fontId="0" fillId="2" borderId="4" xfId="2" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="2" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="4" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="164" fontId="0" fillId="2" borderId="1" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="2" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="3" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="4" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="3" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="3" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="9" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="12" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="2" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="2" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="2" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="2" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="2" borderId="12" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="2" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="2" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="2" borderId="11" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
+    <xf numFmtId="0" fontId="1" fillId="3" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="3" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="2" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
@@ -772,182 +919,35 @@
     <xf numFmtId="0" fontId="0" fillId="2" borderId="4" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="49" fontId="4" fillId="0" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="49" fontId="4" fillId="0" borderId="8" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="49" fontId="4" fillId="0" borderId="12" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="49" fontId="4" fillId="0" borderId="6" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="49" fontId="4" fillId="0" borderId="11" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="49" fontId="4" fillId="2" borderId="7" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="49" fontId="4" fillId="2" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="49" fontId="4" fillId="2" borderId="8" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="49" fontId="4" fillId="2" borderId="9" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="49" fontId="4" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="49" fontId="4" fillId="2" borderId="12" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="49" fontId="4" fillId="2" borderId="10" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="49" fontId="4" fillId="2" borderId="6" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="49" fontId="4" fillId="2" borderId="11" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="2" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="3" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="4" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="164" fontId="0" fillId="2" borderId="2" xfId="2" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="164" fontId="0" fillId="2" borderId="4" xfId="2" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="9" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="12" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="2" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="2" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="2" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="2" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="2" borderId="12" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="2" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="2" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="2" borderId="11" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="2" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="4" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="165" fontId="0" fillId="2" borderId="1" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="49" fontId="4" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="top"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="1" fillId="3" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="1" fillId="3" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="3" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="3" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="3" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
     <xf numFmtId="0" fontId="1" fillId="3" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="13" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="14" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="15" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="16" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="17" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="18" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="19" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="20" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="2" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="3" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="49" fontId="4" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="4" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
+    <xf numFmtId="49" fontId="4" fillId="2" borderId="7" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="49" fontId="4" fillId="2" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="49" fontId="4" fillId="2" borderId="8" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="49" fontId="4" fillId="2" borderId="9" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="49" fontId="4" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="49" fontId="4" fillId="2" borderId="12" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="49" fontId="4" fillId="2" borderId="10" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="49" fontId="4" fillId="2" borderId="6" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="49" fontId="4" fillId="2" borderId="11" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="3">
@@ -1369,19 +1369,19 @@
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
   <dimension ref="A1:L34"/>
-  <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="14.4" x14ac:dyDescent="0.55000000000000004"/>
   <cols>
-    <col min="1" max="1" width="21.5" customWidth="1"/>
-    <col min="4" max="4" width="6.1640625" customWidth="1"/>
-    <col min="7" max="7" width="26.1640625" customWidth="1"/>
-    <col min="8" max="8" width="7.83203125" customWidth="1"/>
-    <col min="9" max="9" width="8.83203125" customWidth="1"/>
-    <col min="10" max="10" width="13.83203125" customWidth="1"/>
-    <col min="11" max="11" width="3.5" customWidth="1"/>
-    <col min="12" max="12" width="12.83203125" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="21.47265625" customWidth="1"/>
+    <col min="4" max="4" width="6.15625" customWidth="1"/>
+    <col min="7" max="7" width="26.15625" customWidth="1"/>
+    <col min="8" max="8" width="7.83984375" customWidth="1"/>
+    <col min="9" max="9" width="8.83984375" customWidth="1"/>
+    <col min="10" max="10" width="13.83984375" customWidth="1"/>
+    <col min="11" max="11" width="3.47265625" customWidth="1"/>
+    <col min="12" max="12" width="12.83984375" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:10" x14ac:dyDescent="0.2">
+    <row r="1" spans="1:10" x14ac:dyDescent="0.55000000000000004">
       <c r="A1" s="1"/>
       <c r="B1" s="1"/>
       <c r="C1" s="1"/>
@@ -1393,7 +1393,7 @@
       <c r="I1" s="1"/>
       <c r="J1" s="1"/>
     </row>
-    <row r="2" spans="1:10" x14ac:dyDescent="0.2">
+    <row r="2" spans="1:10" x14ac:dyDescent="0.55000000000000004">
       <c r="A2" s="1"/>
       <c r="B2" s="1"/>
       <c r="C2" s="1"/>
@@ -1405,7 +1405,7 @@
       <c r="I2" s="1"/>
       <c r="J2" s="1"/>
     </row>
-    <row r="3" spans="1:10" x14ac:dyDescent="0.2">
+    <row r="3" spans="1:10" x14ac:dyDescent="0.55000000000000004">
       <c r="A3" s="1"/>
       <c r="B3" s="1"/>
       <c r="C3" s="1"/>
@@ -1417,27 +1417,27 @@
       <c r="I3" s="1"/>
       <c r="J3" s="1"/>
     </row>
-    <row r="4" spans="1:10" x14ac:dyDescent="0.2">
-      <c r="B4" s="54"/>
-      <c r="C4" s="54"/>
-      <c r="D4" s="54"/>
-      <c r="E4" s="54"/>
+    <row r="4" spans="1:10" x14ac:dyDescent="0.55000000000000004">
+      <c r="B4" s="46"/>
+      <c r="C4" s="46"/>
+      <c r="D4" s="46"/>
+      <c r="E4" s="46"/>
       <c r="F4" s="1"/>
-      <c r="G4" s="60" t="s">
+      <c r="G4" s="21" t="s">
         <v>7</v>
       </c>
-      <c r="H4" s="55" t="s">
+      <c r="H4" s="47" t="s">
         <v>8</v>
       </c>
-      <c r="I4" s="55"/>
-      <c r="J4" s="55"/>
-    </row>
-    <row r="5" spans="1:10" x14ac:dyDescent="0.2">
-      <c r="A5" s="60" t="s">
+      <c r="I4" s="47"/>
+      <c r="J4" s="47"/>
+    </row>
+    <row r="5" spans="1:10" x14ac:dyDescent="0.55000000000000004">
+      <c r="A5" s="21" t="s">
         <v>9</v>
       </c>
       <c r="B5" s="3" t="s">
-        <v>122</v>
+        <v>121</v>
       </c>
       <c r="C5" s="1"/>
       <c r="D5" s="1"/>
@@ -1448,12 +1448,12 @@
       <c r="I5" s="1"/>
       <c r="J5" s="1"/>
     </row>
-    <row r="6" spans="1:10" x14ac:dyDescent="0.2">
-      <c r="A6" s="60" t="s">
+    <row r="6" spans="1:10" x14ac:dyDescent="0.55000000000000004">
+      <c r="A6" s="21" t="s">
+        <v>122</v>
+      </c>
+      <c r="B6" s="3" t="s">
         <v>123</v>
-      </c>
-      <c r="B6" s="3" t="s">
-        <v>124</v>
       </c>
       <c r="C6" s="1"/>
       <c r="D6" s="1"/>
@@ -1464,168 +1464,168 @@
       <c r="I6" s="1"/>
       <c r="J6" s="1"/>
     </row>
-    <row r="7" spans="1:10" x14ac:dyDescent="0.2">
-      <c r="A7" s="60" t="s">
+    <row r="7" spans="1:10" x14ac:dyDescent="0.55000000000000004">
+      <c r="A7" s="21" t="s">
         <v>73</v>
       </c>
-      <c r="B7" s="78" t="s">
+      <c r="B7" s="33" t="s">
         <v>110</v>
       </c>
-      <c r="C7" s="79"/>
-      <c r="D7" s="79"/>
-      <c r="E7" s="79"/>
-      <c r="F7" s="79"/>
-      <c r="G7" s="81"/>
-      <c r="H7" s="21" t="s">
+      <c r="C7" s="34"/>
+      <c r="D7" s="34"/>
+      <c r="E7" s="34"/>
+      <c r="F7" s="34"/>
+      <c r="G7" s="35"/>
+      <c r="H7" s="36" t="s">
         <v>72</v>
       </c>
-      <c r="I7" s="21"/>
-      <c r="J7" s="22"/>
-    </row>
-    <row r="8" spans="1:10" ht="15" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A8" s="61" t="s">
+      <c r="I7" s="36"/>
+      <c r="J7" s="37"/>
+    </row>
+    <row r="8" spans="1:10" ht="15" customHeight="1" x14ac:dyDescent="0.55000000000000004">
+      <c r="A8" s="22" t="s">
         <v>67</v>
       </c>
-      <c r="B8" s="40" t="s">
+      <c r="B8" s="54" t="s">
         <v>111</v>
       </c>
-      <c r="C8" s="41"/>
-      <c r="D8" s="41"/>
-      <c r="E8" s="41"/>
-      <c r="F8" s="41"/>
-      <c r="G8" s="42"/>
-      <c r="H8" s="80"/>
-      <c r="I8" s="80"/>
-      <c r="J8" s="23"/>
-    </row>
-    <row r="9" spans="1:10" x14ac:dyDescent="0.2">
-      <c r="A9" s="62" t="s">
+      <c r="C8" s="55"/>
+      <c r="D8" s="55"/>
+      <c r="E8" s="55"/>
+      <c r="F8" s="55"/>
+      <c r="G8" s="56"/>
+      <c r="H8" s="38"/>
+      <c r="I8" s="38"/>
+      <c r="J8" s="39"/>
+    </row>
+    <row r="9" spans="1:10" x14ac:dyDescent="0.55000000000000004">
+      <c r="A9" s="51" t="s">
         <v>87</v>
       </c>
-      <c r="B9" s="43" t="s">
+      <c r="B9" s="57" t="s">
         <v>109</v>
       </c>
-      <c r="C9" s="44"/>
-      <c r="D9" s="44"/>
-      <c r="E9" s="44"/>
-      <c r="F9" s="44"/>
-      <c r="G9" s="45"/>
-      <c r="H9" s="80"/>
-      <c r="I9" s="80"/>
-      <c r="J9" s="23"/>
-    </row>
-    <row r="10" spans="1:10" x14ac:dyDescent="0.2">
-      <c r="A10" s="63"/>
-      <c r="B10" s="46"/>
-      <c r="C10" s="47"/>
-      <c r="D10" s="47"/>
-      <c r="E10" s="47"/>
-      <c r="F10" s="47"/>
-      <c r="G10" s="48"/>
-      <c r="H10" s="80"/>
-      <c r="I10" s="80"/>
-      <c r="J10" s="23"/>
-    </row>
-    <row r="11" spans="1:10" x14ac:dyDescent="0.2">
-      <c r="A11" s="64"/>
-      <c r="B11" s="49"/>
-      <c r="C11" s="50"/>
-      <c r="D11" s="50"/>
-      <c r="E11" s="50"/>
-      <c r="F11" s="50"/>
-      <c r="G11" s="51"/>
-      <c r="H11" s="80"/>
-      <c r="I11" s="80"/>
-      <c r="J11" s="23"/>
-    </row>
-    <row r="12" spans="1:10" x14ac:dyDescent="0.2">
-      <c r="A12" s="60" t="s">
+      <c r="C9" s="58"/>
+      <c r="D9" s="58"/>
+      <c r="E9" s="58"/>
+      <c r="F9" s="58"/>
+      <c r="G9" s="59"/>
+      <c r="H9" s="38"/>
+      <c r="I9" s="38"/>
+      <c r="J9" s="39"/>
+    </row>
+    <row r="10" spans="1:10" x14ac:dyDescent="0.55000000000000004">
+      <c r="A10" s="52"/>
+      <c r="B10" s="60"/>
+      <c r="C10" s="61"/>
+      <c r="D10" s="61"/>
+      <c r="E10" s="61"/>
+      <c r="F10" s="61"/>
+      <c r="G10" s="62"/>
+      <c r="H10" s="38"/>
+      <c r="I10" s="38"/>
+      <c r="J10" s="39"/>
+    </row>
+    <row r="11" spans="1:10" x14ac:dyDescent="0.55000000000000004">
+      <c r="A11" s="53"/>
+      <c r="B11" s="63"/>
+      <c r="C11" s="64"/>
+      <c r="D11" s="64"/>
+      <c r="E11" s="64"/>
+      <c r="F11" s="64"/>
+      <c r="G11" s="65"/>
+      <c r="H11" s="38"/>
+      <c r="I11" s="38"/>
+      <c r="J11" s="39"/>
+    </row>
+    <row r="12" spans="1:10" x14ac:dyDescent="0.55000000000000004">
+      <c r="A12" s="21" t="s">
         <v>68</v>
       </c>
-      <c r="B12" s="18" t="s">
+      <c r="B12" s="69" t="s">
         <v>14</v>
       </c>
-      <c r="C12" s="19"/>
-      <c r="D12" s="19"/>
-      <c r="E12" s="19"/>
-      <c r="F12" s="19"/>
-      <c r="G12" s="20"/>
-      <c r="H12" s="24"/>
-      <c r="I12" s="24"/>
-      <c r="J12" s="25"/>
-    </row>
-    <row r="13" spans="1:10" x14ac:dyDescent="0.2">
-      <c r="A13" s="58" t="s">
+      <c r="C12" s="70"/>
+      <c r="D12" s="70"/>
+      <c r="E12" s="70"/>
+      <c r="F12" s="70"/>
+      <c r="G12" s="71"/>
+      <c r="H12" s="40"/>
+      <c r="I12" s="40"/>
+      <c r="J12" s="41"/>
+    </row>
+    <row r="13" spans="1:10" x14ac:dyDescent="0.55000000000000004">
+      <c r="A13" s="19" t="s">
         <v>69</v>
       </c>
-      <c r="B13" s="18" t="s">
+      <c r="B13" s="69" t="s">
         <v>39</v>
       </c>
-      <c r="C13" s="19"/>
-      <c r="D13" s="19"/>
-      <c r="E13" s="19"/>
-      <c r="F13" s="19"/>
-      <c r="G13" s="20"/>
-      <c r="H13" s="26" t="s">
+      <c r="C13" s="70"/>
+      <c r="D13" s="70"/>
+      <c r="E13" s="70"/>
+      <c r="F13" s="70"/>
+      <c r="G13" s="71"/>
+      <c r="H13" s="73" t="s">
         <v>66</v>
       </c>
-      <c r="I13" s="27"/>
-      <c r="J13" s="28"/>
-    </row>
-    <row r="14" spans="1:10" x14ac:dyDescent="0.2">
-      <c r="A14" s="58" t="s">
+      <c r="I13" s="74"/>
+      <c r="J13" s="75"/>
+    </row>
+    <row r="14" spans="1:10" x14ac:dyDescent="0.55000000000000004">
+      <c r="A14" s="19" t="s">
         <v>70</v>
       </c>
-      <c r="B14" s="18" t="s">
+      <c r="B14" s="69" t="s">
         <v>107</v>
       </c>
-      <c r="C14" s="19"/>
-      <c r="D14" s="19"/>
-      <c r="E14" s="19"/>
-      <c r="F14" s="19"/>
-      <c r="G14" s="20"/>
-      <c r="H14" s="29"/>
-      <c r="I14" s="30"/>
-      <c r="J14" s="31"/>
-    </row>
-    <row r="15" spans="1:10" x14ac:dyDescent="0.2">
-      <c r="A15" s="58" t="s">
+      <c r="C14" s="70"/>
+      <c r="D14" s="70"/>
+      <c r="E14" s="70"/>
+      <c r="F14" s="70"/>
+      <c r="G14" s="71"/>
+      <c r="H14" s="76"/>
+      <c r="I14" s="77"/>
+      <c r="J14" s="78"/>
+    </row>
+    <row r="15" spans="1:10" x14ac:dyDescent="0.55000000000000004">
+      <c r="A15" s="19" t="s">
         <v>71</v>
       </c>
-      <c r="B15" s="18" t="s">
+      <c r="B15" s="69" t="s">
         <v>102</v>
       </c>
-      <c r="C15" s="19"/>
-      <c r="D15" s="19"/>
-      <c r="E15" s="19"/>
-      <c r="F15" s="19"/>
-      <c r="G15" s="20"/>
-      <c r="H15" s="32"/>
-      <c r="I15" s="33"/>
-      <c r="J15" s="34"/>
-    </row>
-    <row r="16" spans="1:10" x14ac:dyDescent="0.2">
-      <c r="A16" s="58" t="s">
+      <c r="C15" s="70"/>
+      <c r="D15" s="70"/>
+      <c r="E15" s="70"/>
+      <c r="F15" s="70"/>
+      <c r="G15" s="71"/>
+      <c r="H15" s="79"/>
+      <c r="I15" s="80"/>
+      <c r="J15" s="81"/>
+    </row>
+    <row r="16" spans="1:10" x14ac:dyDescent="0.55000000000000004">
+      <c r="A16" s="19" t="s">
         <v>114</v>
       </c>
-      <c r="B16" s="58" t="s">
+      <c r="B16" s="19" t="s">
         <v>115</v>
       </c>
-      <c r="C16" s="56"/>
-      <c r="D16" s="56"/>
-      <c r="E16" s="56"/>
-      <c r="F16" s="56"/>
-      <c r="G16" s="56"/>
-      <c r="H16" s="57"/>
-      <c r="I16" s="57"/>
-      <c r="J16" s="57"/>
-    </row>
-    <row r="17" spans="1:12" x14ac:dyDescent="0.2">
-      <c r="A17" s="58" t="s">
+      <c r="C16" s="18"/>
+      <c r="D16" s="18"/>
+      <c r="E16" s="18"/>
+      <c r="F16" s="18"/>
+      <c r="G16" s="18"/>
+      <c r="H16" s="17"/>
+      <c r="I16" s="17"/>
+      <c r="J16" s="17"/>
+    </row>
+    <row r="17" spans="1:12" x14ac:dyDescent="0.55000000000000004">
+      <c r="A17" s="19" t="s">
         <v>116</v>
       </c>
-      <c r="B17" s="59" t="s">
-        <v>117</v>
+      <c r="B17" s="20" t="s">
+        <v>124</v>
       </c>
       <c r="C17" s="1"/>
       <c r="D17" s="1"/>
@@ -1636,12 +1636,12 @@
       <c r="I17" s="1"/>
       <c r="J17" s="1"/>
     </row>
-    <row r="18" spans="1:12" x14ac:dyDescent="0.2">
-      <c r="A18" s="58" t="s">
-        <v>118</v>
-      </c>
-      <c r="B18" s="59" t="s">
+    <row r="18" spans="1:12" x14ac:dyDescent="0.55000000000000004">
+      <c r="A18" s="19" t="s">
         <v>117</v>
+      </c>
+      <c r="B18" s="20" t="s">
+        <v>119</v>
       </c>
       <c r="C18" s="1"/>
       <c r="D18" s="1"/>
@@ -1652,12 +1652,12 @@
       <c r="I18" s="1"/>
       <c r="J18" s="1"/>
     </row>
-    <row r="19" spans="1:12" x14ac:dyDescent="0.2">
-      <c r="A19" s="58" t="s">
-        <v>119</v>
-      </c>
-      <c r="B19" s="59" t="s">
-        <v>120</v>
+    <row r="19" spans="1:12" x14ac:dyDescent="0.55000000000000004">
+      <c r="A19" s="19" t="s">
+        <v>118</v>
+      </c>
+      <c r="B19" s="20" t="s">
+        <v>124</v>
       </c>
       <c r="C19" s="1"/>
       <c r="D19" s="1"/>
@@ -1668,7 +1668,7 @@
       <c r="I19" s="1"/>
       <c r="J19" s="1"/>
     </row>
-    <row r="20" spans="1:12" x14ac:dyDescent="0.2">
+    <row r="20" spans="1:12" x14ac:dyDescent="0.55000000000000004">
       <c r="A20" s="1"/>
       <c r="B20" s="3"/>
       <c r="C20" s="1"/>
@@ -1680,128 +1680,128 @@
       <c r="I20" s="1"/>
       <c r="J20" s="1"/>
     </row>
-    <row r="21" spans="1:12" x14ac:dyDescent="0.2">
-      <c r="A21" s="65" t="s">
+    <row r="21" spans="1:12" x14ac:dyDescent="0.55000000000000004">
+      <c r="A21" s="23" t="s">
         <v>0</v>
       </c>
-      <c r="B21" s="65" t="s">
+      <c r="B21" s="23" t="s">
         <v>1</v>
       </c>
-      <c r="C21" s="66" t="s">
+      <c r="C21" s="67" t="s">
         <v>2</v>
       </c>
-      <c r="D21" s="67"/>
-      <c r="E21" s="66" t="s">
+      <c r="D21" s="68"/>
+      <c r="E21" s="67" t="s">
         <v>3</v>
       </c>
-      <c r="F21" s="68"/>
-      <c r="G21" s="67"/>
-      <c r="H21" s="66" t="s">
+      <c r="F21" s="72"/>
+      <c r="G21" s="68"/>
+      <c r="H21" s="67" t="s">
         <v>4</v>
       </c>
-      <c r="I21" s="67"/>
-      <c r="J21" s="65" t="s">
+      <c r="I21" s="68"/>
+      <c r="J21" s="23" t="s">
         <v>5</v>
       </c>
     </row>
-    <row r="22" spans="1:12" ht="40.75" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="22" spans="1:12" ht="40.75" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A22" s="16">
         <v>84101501</v>
       </c>
       <c r="B22" s="13">
         <v>1</v>
       </c>
-      <c r="C22" s="52" t="s">
+      <c r="C22" s="44" t="s">
         <v>112</v>
       </c>
-      <c r="D22" s="53"/>
-      <c r="E22" s="35" t="s">
+      <c r="D22" s="45"/>
+      <c r="E22" s="48" t="s">
         <v>113</v>
       </c>
-      <c r="F22" s="36"/>
-      <c r="G22" s="37"/>
-      <c r="H22" s="38">
+      <c r="F22" s="49"/>
+      <c r="G22" s="50"/>
+      <c r="H22" s="42">
         <v>22500</v>
       </c>
-      <c r="I22" s="39"/>
+      <c r="I22" s="43"/>
       <c r="J22" s="15">
         <f t="shared" ref="J22:J26" si="0">B22*H22</f>
         <v>22500</v>
       </c>
     </row>
-    <row r="23" spans="1:12" ht="14.5" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="23" spans="1:12" ht="14.5" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A23" s="12"/>
       <c r="B23" s="13"/>
-      <c r="C23" s="52"/>
-      <c r="D23" s="53"/>
-      <c r="E23" s="35"/>
-      <c r="F23" s="36"/>
-      <c r="G23" s="37"/>
-      <c r="H23" s="38"/>
-      <c r="I23" s="39"/>
+      <c r="C23" s="44"/>
+      <c r="D23" s="45"/>
+      <c r="E23" s="48"/>
+      <c r="F23" s="49"/>
+      <c r="G23" s="50"/>
+      <c r="H23" s="42"/>
+      <c r="I23" s="43"/>
       <c r="J23" s="15">
         <f t="shared" si="0"/>
         <v>0</v>
       </c>
     </row>
-    <row r="24" spans="1:12" ht="14.5" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="24" spans="1:12" ht="14.5" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A24" s="12"/>
       <c r="B24" s="13"/>
-      <c r="C24" s="52"/>
-      <c r="D24" s="53"/>
-      <c r="E24" s="35"/>
-      <c r="F24" s="36"/>
-      <c r="G24" s="37"/>
-      <c r="H24" s="38"/>
-      <c r="I24" s="39"/>
+      <c r="C24" s="44"/>
+      <c r="D24" s="45"/>
+      <c r="E24" s="48"/>
+      <c r="F24" s="49"/>
+      <c r="G24" s="50"/>
+      <c r="H24" s="42"/>
+      <c r="I24" s="43"/>
       <c r="J24" s="15">
         <f t="shared" si="0"/>
         <v>0</v>
       </c>
     </row>
-    <row r="25" spans="1:12" ht="14.5" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="25" spans="1:12" ht="14.5" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A25" s="12"/>
       <c r="B25" s="13"/>
-      <c r="C25" s="52"/>
-      <c r="D25" s="53"/>
-      <c r="E25" s="35"/>
-      <c r="F25" s="36"/>
-      <c r="G25" s="37"/>
-      <c r="H25" s="38"/>
-      <c r="I25" s="39"/>
+      <c r="C25" s="44"/>
+      <c r="D25" s="45"/>
+      <c r="E25" s="48"/>
+      <c r="F25" s="49"/>
+      <c r="G25" s="50"/>
+      <c r="H25" s="42"/>
+      <c r="I25" s="43"/>
       <c r="J25" s="15">
         <f t="shared" si="0"/>
         <v>0</v>
       </c>
     </row>
-    <row r="26" spans="1:12" ht="14.5" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="26" spans="1:12" ht="14.5" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A26" s="12"/>
       <c r="B26" s="13"/>
-      <c r="C26" s="52"/>
-      <c r="D26" s="53"/>
-      <c r="E26" s="35"/>
-      <c r="F26" s="36"/>
-      <c r="G26" s="37"/>
-      <c r="H26" s="38"/>
-      <c r="I26" s="39"/>
+      <c r="C26" s="44"/>
+      <c r="D26" s="45"/>
+      <c r="E26" s="48"/>
+      <c r="F26" s="49"/>
+      <c r="G26" s="50"/>
+      <c r="H26" s="42"/>
+      <c r="I26" s="43"/>
       <c r="J26" s="15">
         <f t="shared" si="0"/>
         <v>0</v>
       </c>
     </row>
-    <row r="27" spans="1:12" x14ac:dyDescent="0.2">
+    <row r="27" spans="1:12" x14ac:dyDescent="0.55000000000000004">
       <c r="A27" s="1"/>
       <c r="B27" s="1"/>
-      <c r="C27" s="17"/>
-      <c r="D27" s="17"/>
-      <c r="E27" s="17"/>
-      <c r="F27" s="17"/>
-      <c r="G27" s="17"/>
-      <c r="H27" s="17"/>
+      <c r="C27" s="66"/>
+      <c r="D27" s="66"/>
+      <c r="E27" s="66"/>
+      <c r="F27" s="66"/>
+      <c r="G27" s="66"/>
+      <c r="H27" s="66"/>
       <c r="I27" s="1"/>
       <c r="J27" s="1"/>
     </row>
-    <row r="28" spans="1:12" x14ac:dyDescent="0.2">
+    <row r="28" spans="1:12" x14ac:dyDescent="0.55000000000000004">
       <c r="A28" s="1"/>
       <c r="B28" s="1"/>
       <c r="C28" s="1"/>
@@ -1820,7 +1820,7 @@
       <c r="K28" s="10"/>
       <c r="L28" s="11"/>
     </row>
-    <row r="29" spans="1:12" x14ac:dyDescent="0.2">
+    <row r="29" spans="1:12" x14ac:dyDescent="0.55000000000000004">
       <c r="A29" s="1"/>
       <c r="B29" s="1"/>
       <c r="C29" s="1"/>
@@ -1838,7 +1838,7 @@
       </c>
       <c r="L29" s="14"/>
     </row>
-    <row r="30" spans="1:12" x14ac:dyDescent="0.2">
+    <row r="30" spans="1:12" x14ac:dyDescent="0.55000000000000004">
       <c r="F30" s="1"/>
       <c r="G30" s="1"/>
       <c r="H30" s="1"/>
@@ -1850,70 +1850,57 @@
         <v>26100</v>
       </c>
     </row>
-    <row r="31" spans="1:12" ht="16" thickBot="1" x14ac:dyDescent="0.25">
+    <row r="31" spans="1:12" ht="14.7" thickBot="1" x14ac:dyDescent="0.6">
       <c r="F31" s="9"/>
       <c r="G31" s="9"/>
       <c r="H31" s="1"/>
       <c r="I31" s="1"/>
       <c r="J31" s="1"/>
     </row>
-    <row r="32" spans="1:12" x14ac:dyDescent="0.2">
-      <c r="A32" s="61" t="s">
-        <v>121</v>
-      </c>
-      <c r="B32" s="69"/>
-      <c r="C32" s="70"/>
-      <c r="D32" s="70"/>
-      <c r="E32" s="70"/>
-      <c r="F32" s="70"/>
-      <c r="G32" s="70"/>
-      <c r="H32" s="70"/>
-      <c r="I32" s="70"/>
-      <c r="J32" s="71"/>
-    </row>
-    <row r="33" spans="2:10" x14ac:dyDescent="0.2">
-      <c r="B33" s="72"/>
-      <c r="C33" s="73"/>
-      <c r="D33" s="73"/>
-      <c r="E33" s="73"/>
-      <c r="F33" s="73"/>
-      <c r="G33" s="73"/>
-      <c r="H33" s="73"/>
-      <c r="I33" s="73"/>
-      <c r="J33" s="74"/>
-    </row>
-    <row r="34" spans="2:10" ht="16" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="B34" s="75"/>
-      <c r="C34" s="76"/>
-      <c r="D34" s="76"/>
-      <c r="E34" s="76"/>
-      <c r="F34" s="76"/>
-      <c r="G34" s="76"/>
-      <c r="H34" s="76"/>
-      <c r="I34" s="76"/>
-      <c r="J34" s="77"/>
+    <row r="32" spans="1:12" x14ac:dyDescent="0.55000000000000004">
+      <c r="A32" s="22" t="s">
+        <v>120</v>
+      </c>
+      <c r="B32" s="24"/>
+      <c r="C32" s="25"/>
+      <c r="D32" s="25"/>
+      <c r="E32" s="25"/>
+      <c r="F32" s="25"/>
+      <c r="G32" s="25"/>
+      <c r="H32" s="25"/>
+      <c r="I32" s="25"/>
+      <c r="J32" s="26"/>
+    </row>
+    <row r="33" spans="2:10" x14ac:dyDescent="0.55000000000000004">
+      <c r="B33" s="27"/>
+      <c r="C33" s="28"/>
+      <c r="D33" s="28"/>
+      <c r="E33" s="28"/>
+      <c r="F33" s="28"/>
+      <c r="G33" s="28"/>
+      <c r="H33" s="28"/>
+      <c r="I33" s="28"/>
+      <c r="J33" s="29"/>
+    </row>
+    <row r="34" spans="2:10" ht="14.7" thickBot="1" x14ac:dyDescent="0.6">
+      <c r="B34" s="30"/>
+      <c r="C34" s="31"/>
+      <c r="D34" s="31"/>
+      <c r="E34" s="31"/>
+      <c r="F34" s="31"/>
+      <c r="G34" s="31"/>
+      <c r="H34" s="31"/>
+      <c r="I34" s="31"/>
+      <c r="J34" s="32"/>
     </row>
   </sheetData>
   <mergeCells count="32">
-    <mergeCell ref="B32:J34"/>
-    <mergeCell ref="B7:G7"/>
-    <mergeCell ref="H7:J12"/>
-    <mergeCell ref="H26:I26"/>
-    <mergeCell ref="C24:D24"/>
-    <mergeCell ref="C25:D25"/>
-    <mergeCell ref="C26:D26"/>
-    <mergeCell ref="B4:E4"/>
-    <mergeCell ref="H4:J4"/>
-    <mergeCell ref="C23:D23"/>
-    <mergeCell ref="E23:G23"/>
-    <mergeCell ref="H23:I23"/>
     <mergeCell ref="A9:A11"/>
     <mergeCell ref="B8:G8"/>
     <mergeCell ref="B9:G11"/>
     <mergeCell ref="C22:D22"/>
     <mergeCell ref="H22:I22"/>
     <mergeCell ref="E22:G22"/>
-    <mergeCell ref="C27:H27"/>
     <mergeCell ref="C21:D21"/>
     <mergeCell ref="H21:I21"/>
     <mergeCell ref="B13:G13"/>
@@ -1922,6 +1909,19 @@
     <mergeCell ref="E21:G21"/>
     <mergeCell ref="B12:G12"/>
     <mergeCell ref="H13:J15"/>
+    <mergeCell ref="B4:E4"/>
+    <mergeCell ref="H4:J4"/>
+    <mergeCell ref="C23:D23"/>
+    <mergeCell ref="E23:G23"/>
+    <mergeCell ref="H23:I23"/>
+    <mergeCell ref="B32:J34"/>
+    <mergeCell ref="B7:G7"/>
+    <mergeCell ref="H7:J12"/>
+    <mergeCell ref="H26:I26"/>
+    <mergeCell ref="C24:D24"/>
+    <mergeCell ref="C25:D25"/>
+    <mergeCell ref="C26:D26"/>
+    <mergeCell ref="C27:H27"/>
     <mergeCell ref="E24:G24"/>
     <mergeCell ref="E25:G25"/>
     <mergeCell ref="E26:G26"/>
@@ -1975,15 +1975,15 @@
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
   <dimension ref="A1:G28"/>
-  <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="14.4" x14ac:dyDescent="0.55000000000000004"/>
   <cols>
-    <col min="1" max="1" width="39.5" customWidth="1"/>
-    <col min="3" max="3" width="56.1640625" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="33.83203125" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="87.83203125" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="39.47265625" customWidth="1"/>
+    <col min="3" max="3" width="56.15625" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="33.83984375" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="87.83984375" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="1" spans="1:7" x14ac:dyDescent="0.55000000000000004">
       <c r="A1" t="s">
         <v>13</v>
       </c>
@@ -1997,7 +1997,7 @@
         <v>37</v>
       </c>
     </row>
-    <row r="2" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="2" spans="1:7" x14ac:dyDescent="0.55000000000000004">
       <c r="A2" t="s">
         <v>12</v>
       </c>
@@ -2011,7 +2011,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="3" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="3" spans="1:7" x14ac:dyDescent="0.55000000000000004">
       <c r="A3" t="s">
         <v>75</v>
       </c>
@@ -2025,7 +2025,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="4" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="4" spans="1:7" x14ac:dyDescent="0.55000000000000004">
       <c r="C4" t="s">
         <v>40</v>
       </c>
@@ -2036,7 +2036,7 @@
         <v>16</v>
       </c>
     </row>
-    <row r="5" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="5" spans="1:7" x14ac:dyDescent="0.55000000000000004">
       <c r="A5" t="s">
         <v>10</v>
       </c>
@@ -2050,7 +2050,7 @@
         <v>18</v>
       </c>
     </row>
-    <row r="6" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="6" spans="1:7" x14ac:dyDescent="0.55000000000000004">
       <c r="A6" t="s">
         <v>78</v>
       </c>
@@ -2064,7 +2064,7 @@
         <v>17</v>
       </c>
     </row>
-    <row r="7" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="7" spans="1:7" x14ac:dyDescent="0.55000000000000004">
       <c r="A7" t="s">
         <v>11</v>
       </c>
@@ -2078,7 +2078,7 @@
         <v>19</v>
       </c>
     </row>
-    <row r="8" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="8" spans="1:7" x14ac:dyDescent="0.55000000000000004">
       <c r="A8" t="s">
         <v>91</v>
       </c>
@@ -2092,7 +2092,7 @@
         <v>20</v>
       </c>
     </row>
-    <row r="9" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="9" spans="1:7" x14ac:dyDescent="0.55000000000000004">
       <c r="A9" t="s">
         <v>77</v>
       </c>
@@ -2106,7 +2106,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="10" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="10" spans="1:7" x14ac:dyDescent="0.55000000000000004">
       <c r="A10" t="s">
         <v>85</v>
       </c>
@@ -2120,7 +2120,7 @@
         <v>22</v>
       </c>
     </row>
-    <row r="11" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="11" spans="1:7" x14ac:dyDescent="0.55000000000000004">
       <c r="A11" t="s">
         <v>86</v>
       </c>
@@ -2134,7 +2134,7 @@
         <v>23</v>
       </c>
     </row>
-    <row r="12" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="12" spans="1:7" x14ac:dyDescent="0.55000000000000004">
       <c r="A12" t="s">
         <v>88</v>
       </c>
@@ -2145,7 +2145,7 @@
         <v>24</v>
       </c>
     </row>
-    <row r="13" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="13" spans="1:7" x14ac:dyDescent="0.55000000000000004">
       <c r="A13" t="s">
         <v>89</v>
       </c>
@@ -2156,7 +2156,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="14" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="14" spans="1:7" x14ac:dyDescent="0.55000000000000004">
       <c r="A14" t="s">
         <v>90</v>
       </c>
@@ -2167,7 +2167,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="15" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="15" spans="1:7" x14ac:dyDescent="0.55000000000000004">
       <c r="A15" t="s">
         <v>95</v>
       </c>
@@ -2178,7 +2178,7 @@
         <v>27</v>
       </c>
     </row>
-    <row r="16" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="16" spans="1:7" x14ac:dyDescent="0.55000000000000004">
       <c r="A16" t="s">
         <v>96</v>
       </c>
@@ -2189,7 +2189,7 @@
         <v>28</v>
       </c>
     </row>
-    <row r="17" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="17" spans="1:7" x14ac:dyDescent="0.55000000000000004">
       <c r="A17" t="s">
         <v>97</v>
       </c>
@@ -2200,7 +2200,7 @@
         <v>29</v>
       </c>
     </row>
-    <row r="18" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="18" spans="1:7" x14ac:dyDescent="0.55000000000000004">
       <c r="A18" t="s">
         <v>98</v>
       </c>
@@ -2211,7 +2211,7 @@
         <v>30</v>
       </c>
     </row>
-    <row r="19" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="19" spans="1:7" x14ac:dyDescent="0.55000000000000004">
       <c r="A19" t="s">
         <v>99</v>
       </c>
@@ -2222,7 +2222,7 @@
         <v>31</v>
       </c>
     </row>
-    <row r="20" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="20" spans="1:7" x14ac:dyDescent="0.55000000000000004">
       <c r="A20" t="s">
         <v>100</v>
       </c>
@@ -2233,7 +2233,7 @@
         <v>32</v>
       </c>
     </row>
-    <row r="21" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="21" spans="1:7" x14ac:dyDescent="0.55000000000000004">
       <c r="A21" t="s">
         <v>101</v>
       </c>
@@ -2244,7 +2244,7 @@
         <v>33</v>
       </c>
     </row>
-    <row r="22" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="22" spans="1:7" x14ac:dyDescent="0.55000000000000004">
       <c r="A22" t="s">
         <v>108</v>
       </c>
@@ -2255,7 +2255,7 @@
         <v>34</v>
       </c>
     </row>
-    <row r="23" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="23" spans="1:7" x14ac:dyDescent="0.55000000000000004">
       <c r="E23" t="s">
         <v>82</v>
       </c>
@@ -2263,7 +2263,7 @@
         <v>35</v>
       </c>
     </row>
-    <row r="24" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="24" spans="1:7" x14ac:dyDescent="0.55000000000000004">
       <c r="E24" t="s">
         <v>83</v>
       </c>
@@ -2271,22 +2271,22 @@
         <v>36</v>
       </c>
     </row>
-    <row r="25" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="25" spans="1:7" x14ac:dyDescent="0.55000000000000004">
       <c r="E25" t="s">
         <v>84</v>
       </c>
     </row>
-    <row r="26" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="26" spans="1:7" x14ac:dyDescent="0.55000000000000004">
       <c r="E26" t="s">
         <v>92</v>
       </c>
     </row>
-    <row r="27" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="27" spans="1:7" x14ac:dyDescent="0.55000000000000004">
       <c r="E27" t="s">
         <v>93</v>
       </c>
     </row>
-    <row r="28" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="28" spans="1:7" x14ac:dyDescent="0.55000000000000004">
       <c r="E28" t="s">
         <v>94</v>
       </c>
@@ -2305,15 +2305,15 @@
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{35D63560-B92C-4115-87ED-D53B987A5514}">
   <dimension ref="A1:D2"/>
-  <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="14.4" x14ac:dyDescent="0.55000000000000004"/>
   <cols>
-    <col min="1" max="1" width="15.5" customWidth="1"/>
-    <col min="2" max="2" width="14.5" customWidth="1"/>
-    <col min="3" max="3" width="21.5" customWidth="1"/>
-    <col min="4" max="4" width="18.83203125" customWidth="1"/>
+    <col min="1" max="1" width="15.47265625" customWidth="1"/>
+    <col min="2" max="2" width="14.47265625" customWidth="1"/>
+    <col min="3" max="3" width="21.47265625" customWidth="1"/>
+    <col min="4" max="4" width="18.83984375" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:4" x14ac:dyDescent="0.2">
+    <row r="1" spans="1:4" x14ac:dyDescent="0.55000000000000004">
       <c r="A1" t="s">
         <v>104</v>
       </c>
@@ -2327,7 +2327,7 @@
         <v>106</v>
       </c>
     </row>
-    <row r="2" spans="1:4" x14ac:dyDescent="0.2">
+    <row r="2" spans="1:4" x14ac:dyDescent="0.55000000000000004">
       <c r="A2" t="s">
         <v>102</v>
       </c>

</xml_diff>